<commit_message>
Deploy 65 bespoke client portals: instant 0ms mesh backgrounds, prominent mobile front-page property images, zero demo controls, and updated Excel outreach engine
</commit_message>
<xml_diff>
--- a/Pakistan_Real_Estate_WhatsApp_Outreach_Engine_Upgraded.xlsx
+++ b/Pakistan_Real_Estate_WhatsApp_Outreach_Engine_Upgraded.xlsx
@@ -9968,7 +9968,7 @@
       <c r="S2" s="45" t="inlineStr">
         <is>
           <t>Shukriya sir! Here is the live mobile preview I put together for Three Realtors:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/three-realtors
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -10074,7 +10074,7 @@
       <c r="S3" s="47" t="inlineStr">
         <is>
           <t>Shukriya sir! Here is the live mobile preview I put together for HomeNet Real Estate:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/homenet-real
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -10180,7 +10180,7 @@
       <c r="S4" s="45" t="inlineStr">
         <is>
           <t>Shukriya sir! Here is the live mobile preview I put together for Binferoz Enterprises:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/binferoz-real
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -10286,7 +10286,7 @@
       <c r="S5" s="47" t="inlineStr">
         <is>
           <t>Shukriya Sarim bhai! Here is the live mobile preview I put together for Sarim Raza Estate:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/sarim-raza
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -10392,7 +10392,7 @@
       <c r="S6" s="45" t="inlineStr">
         <is>
           <t>Shukriya Tanveer bhai! Here is the live mobile preview I put together for Jinnah Builders:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/jinnah-builders
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -10498,7 +10498,7 @@
       <c r="S7" s="47" t="inlineStr">
         <is>
           <t>Shukriya Umar bhai! Here is the live mobile preview I put together for Ross Realtors:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/ross-realtors
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -10604,7 +10604,7 @@
       <c r="S8" s="45" t="inlineStr">
         <is>
           <t>Shukriya Adnan bhai! Here is the live mobile preview I put together for Siraat Builders:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/siraat-real
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -10710,7 +10710,7 @@
       <c r="S9" s="47" t="inlineStr">
         <is>
           <t>Shukriya sir! Here is the live mobile preview I put together for Royal Homes:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/royal-homes
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -10816,7 +10816,7 @@
       <c r="S10" s="45" t="inlineStr">
         <is>
           <t>Shukriya sir! Here is the live mobile preview I put together for GFS Builders (Gulshan):
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/gfs-builders
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -10922,7 +10922,7 @@
       <c r="S11" s="47" t="inlineStr">
         <is>
           <t>Shukriya sir! Here is the live mobile preview I put together for AHH Brothers:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/ahh-brothers
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -11028,7 +11028,7 @@
       <c r="S12" s="45" t="inlineStr">
         <is>
           <t>Shukriya sir! Here is the live mobile preview I put together for Lenaar Group:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/lenaar-group
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -11134,7 +11134,7 @@
       <c r="S13" s="47" t="inlineStr">
         <is>
           <t>Shukriya sir! Here is the live mobile preview I put together for Al Hassan Estate:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/al-hassan
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -11240,7 +11240,7 @@
       <c r="S14" s="45" t="inlineStr">
         <is>
           <t>Shukriya Ahmer bhai! Here is the live mobile preview I put together for Matloob Real Estate:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/matloob-real
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -11346,7 +11346,7 @@
       <c r="S15" s="47" t="inlineStr">
         <is>
           <t>Shukriya Ovais bhai! Here is the live mobile preview I put together for Paragon Estate:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/paragon-estate
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -11452,7 +11452,7 @@
       <c r="S16" s="45" t="inlineStr">
         <is>
           <t>Shukriya sir! Here is the live mobile preview I put together for AA Builders:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/aa-builders
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -11558,7 +11558,7 @@
       <c r="S17" s="47" t="inlineStr">
         <is>
           <t>Shukriya sir! Here is the live mobile preview I put together for Anaya Estate:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/anaya-estate
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -11664,7 +11664,7 @@
       <c r="S18" s="45" t="inlineStr">
         <is>
           <t>Shukriya sir! Here is the live mobile preview I put together for Hafiz Builders:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/hafiz-real
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -11770,7 +11770,7 @@
       <c r="S19" s="47" t="inlineStr">
         <is>
           <t>Shukriya sir! Here is the live mobile preview I put together for M.A Estates:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/m-a
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -11876,7 +11876,7 @@
       <c r="S20" s="45" t="inlineStr">
         <is>
           <t>Shukriya Sajid Aslam sahib! Here is the live mobile preview I put together for 92 Al Qaswa Builders:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/92-al
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -11982,7 +11982,7 @@
       <c r="S21" s="47" t="inlineStr">
         <is>
           <t>Shukriya Asif Shamim sahib! Here is the live mobile preview I put together for 3G Builders:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/3g-builders
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -12088,7 +12088,7 @@
       <c r="S22" s="45" t="inlineStr">
         <is>
           <t>Shukriya Faisal Sherazee sahib! Here is the live mobile preview I put together for A.E &amp; H Builders:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/a-e
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -12194,7 +12194,7 @@
       <c r="S23" s="47" t="inlineStr">
         <is>
           <t>Shukriya Haya Khan sahib! Here is the live mobile preview I put together for Abraaj Gold Builders:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/abraaj-gold
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -12300,7 +12300,7 @@
       <c r="S24" s="45" t="inlineStr">
         <is>
           <t>Shukriya Umair Saghir sahib! Here is the live mobile preview I put together for Ahmed Mustufa Builders:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/ahmed-mustufa
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -12406,7 +12406,7 @@
       <c r="S25" s="47" t="inlineStr">
         <is>
           <t>Shukriya Amir Raza sahib! Here is the live mobile preview I put together for Al-Kafeel Builders:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/al-kafeel
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -12512,7 +12512,7 @@
       <c r="S26" s="45" t="inlineStr">
         <is>
           <t>Shukriya Ziad Khalid sahib! Here is the live mobile preview I put together for Al-Khalid Builders:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/al-khalid
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -12618,7 +12618,7 @@
       <c r="S27" s="47" t="inlineStr">
         <is>
           <t>Shukriya Umer Mukhtar sahib! Here is the live mobile preview I put together for Al-Mukhtar Builders:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/al-mukhtar
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -12724,7 +12724,7 @@
       <c r="S28" s="45" t="inlineStr">
         <is>
           <t>Shukriya Imran Siddiqui sahib! Here is the live mobile preview I put together for Al-Qasar Builders:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/al-qasar
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -12830,7 +12830,7 @@
       <c r="S29" s="47" t="inlineStr">
         <is>
           <t>Shukriya sir! Here is the live mobile preview I put together for Lodhi Builders:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/lodhi-builders
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -12936,7 +12936,7 @@
       <c r="S30" s="45" t="inlineStr">
         <is>
           <t>Shukriya sir! Here is the live mobile preview I put together for Deal Land Builders:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/deal-land
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -13042,7 +13042,7 @@
       <c r="S31" s="47" t="inlineStr">
         <is>
           <t>Shukriya Waqar bhai! Here is the live mobile preview I put together for Haris Real Estate:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/haris-real
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -13148,7 +13148,7 @@
       <c r="S32" s="45" t="inlineStr">
         <is>
           <t>Shukriya sir! Here is the live mobile preview I put together for Property Master (PMB):
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/property-master
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -13254,7 +13254,7 @@
       <c r="S33" s="47" t="inlineStr">
         <is>
           <t>Shukriya Ghulam Muhaudin sahib! Here is the live mobile preview I put together for GM Developers:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/gm-real
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -13360,7 +13360,7 @@
       <c r="S34" s="45" t="inlineStr">
         <is>
           <t>Shukriya sir! Here is the live mobile preview I put together for Zahid Estate:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/zahid-estate
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -13466,7 +13466,7 @@
       <c r="S35" s="47" t="inlineStr">
         <is>
           <t>Shukriya sir! Here is the live mobile preview I put together for NM Associates:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/nm-associates
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -13572,7 +13572,7 @@
       <c r="S36" s="45" t="inlineStr">
         <is>
           <t>Shukriya sir! Here is the live mobile preview I put together for Harum Estate:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/harum-estate
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -13678,7 +13678,7 @@
       <c r="S37" s="47" t="inlineStr">
         <is>
           <t>Shukriya sir! Here is the live mobile preview I put together for Hamd Estate:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/hamd-estate
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -13784,7 +13784,7 @@
       <c r="S38" s="45" t="inlineStr">
         <is>
           <t>Shukriya sir! Here is the live mobile preview I put together for Kareem Builders:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/kareem-real
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -13890,7 +13890,7 @@
       <c r="S39" s="47" t="inlineStr">
         <is>
           <t>Shukriya sir! Here is the live mobile preview I put together for Ali Baba Estate:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/ali-baba
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -13996,7 +13996,7 @@
       <c r="S40" s="45" t="inlineStr">
         <is>
           <t>Shukriya Suleman Habib sahib! Here is the live mobile preview I put together for Al-Habib Builders:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/al-habib
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -14102,7 +14102,7 @@
       <c r="S41" s="47" t="inlineStr">
         <is>
           <t>Shukriya sir! Here is the live mobile preview I put together for AlRehman Property:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/alrehman-property
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -14208,7 +14208,7 @@
       <c r="S42" s="45" t="inlineStr">
         <is>
           <t>Shukriya sir! Here is the live mobile preview I put together for Gold Bricks Builders:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/gold-bricks
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -14314,7 +14314,7 @@
       <c r="S43" s="47" t="inlineStr">
         <is>
           <t>Shukriya Mian Umer sahib! Here is the live mobile preview I put together for Akbar Groups:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/akbar-real
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -14420,7 +14420,7 @@
       <c r="S44" s="45" t="inlineStr">
         <is>
           <t>Shukriya sir! Here is the live mobile preview I put together for Top Value Associates:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/top-value
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -14526,7 +14526,7 @@
       <c r="S45" s="47" t="inlineStr">
         <is>
           <t>Shukriya sir! Here is the live mobile preview I put together for Land Mark Estate:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/land-mark
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -14632,7 +14632,7 @@
       <c r="S46" s="45" t="inlineStr">
         <is>
           <t>Shukriya Abdul Rauf sahib! Here is the live mobile preview I put together for A.R. Alam Builders:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/a-r
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -14738,7 +14738,7 @@
       <c r="S47" s="47" t="inlineStr">
         <is>
           <t>Shukriya Mohsin bhai! Here is the live mobile preview I put together for Onyx International:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/onyx-international
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -14844,7 +14844,7 @@
       <c r="S48" s="45" t="inlineStr">
         <is>
           <t>Shukriya sir! Here is the live mobile preview I put together for Sultan's Construction:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/sultan-s
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -14950,7 +14950,7 @@
       <c r="S49" s="47" t="inlineStr">
         <is>
           <t>Shukriya sir! Here is the live mobile preview I put together for Imar Associates:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/imar-associates
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -15056,7 +15056,7 @@
       <c r="S50" s="45" t="inlineStr">
         <is>
           <t>Shukriya Engr. Ihtisham sahib! Here is the live mobile preview I put together for Zamung Kor Builders:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/zamung-kor
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -15162,7 +15162,7 @@
       <c r="S51" s="47" t="inlineStr">
         <is>
           <t>Shukriya Mujtaba bhai! Here is the live mobile preview I put together for Prospect Realty:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/prospect-realty
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -15268,7 +15268,7 @@
       <c r="S52" s="45" t="inlineStr">
         <is>
           <t>Shukriya Kaleem Saif sahib! Here is the live mobile preview I put together for Home Land Builders:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/home-land
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -15374,7 +15374,7 @@
       <c r="S53" s="47" t="inlineStr">
         <is>
           <t>Shukriya sir! Here is the live mobile preview I put together for NWR Builders:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/n-w
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -15480,7 +15480,7 @@
       <c r="S54" s="45" t="inlineStr">
         <is>
           <t>Shukriya sir! Here is the live mobile preview I put together for Hayatabad Property:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/hayatabad-property
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -15586,7 +15586,7 @@
       <c r="S55" s="47" t="inlineStr">
         <is>
           <t>Shukriya sir! Here is the live mobile preview I put together for Eshaal Builders:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/eshaal-real
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -15692,7 +15692,7 @@
       <c r="S56" s="45" t="inlineStr">
         <is>
           <t>Shukriya sir! Here is the live mobile preview I put together for 5G Properties:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/5g-properties
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -15798,7 +15798,7 @@
       <c r="S57" s="47" t="inlineStr">
         <is>
           <t>Shukriya Talha bhai! Here is the live mobile preview I put together for Talha Real Estate:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/talha-real
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -15904,7 +15904,7 @@
       <c r="S58" s="45" t="inlineStr">
         <is>
           <t>Shukriya sir! Here is the live mobile preview I put together for Dreams Real Estate:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/dreams-real
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -16010,7 +16010,7 @@
       <c r="S59" s="47" t="inlineStr">
         <is>
           <t>Shukriya Usman Butt sahib! Here is the live mobile preview I put together for Bismillah Estate:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/bismillah-estate
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -16116,7 +16116,7 @@
       <c r="S60" s="45" t="inlineStr">
         <is>
           <t>Shukriya Rizwan Pasha sahib! Here is the live mobile preview I put together for Pasha Estate:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/pasha-estate
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -16222,7 +16222,7 @@
       <c r="S61" s="47" t="inlineStr">
         <is>
           <t>Shukriya sir! Here is the live mobile preview I put together for Modern Homes Builders:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/modern-homes
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -16328,7 +16328,7 @@
       <c r="S62" s="45" t="inlineStr">
         <is>
           <t>Shukriya Shahzeb bhai! Here is the live mobile preview I put together for Falcon Real Estate:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/falcon-real
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -16434,7 +16434,7 @@
       <c r="S63" s="47" t="inlineStr">
         <is>
           <t>Shukriya sir! Here is the live mobile preview I put together for Experts Estate:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/experts-estate
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -16540,7 +16540,7 @@
       <c r="S64" s="45" t="inlineStr">
         <is>
           <t>Shukriya sir! Here is the live mobile preview I put together for Future Builders:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/future-real
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -16646,7 +16646,7 @@
       <c r="S65" s="47" t="inlineStr">
         <is>
           <t>Shukriya sir! Here is the live mobile preview I put together for MA Real Estate:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/ma-realestate
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.
@@ -16752,7 +16752,7 @@
       <c r="S66" s="45" t="inlineStr">
         <is>
           <t>Shukriya sir! Here is the live mobile preview I put together for Real Constructors:
-👉 [INSERT_YOUR_DEMO_LINK_HERE]
+👉 https://real-estate-outreach.pages.dev/real-constructors
 Notice 3 quick things when you tap through it on your phone:
 1. Zero 20MB PDF friction: Buyers see your featured projects, floor plans &amp; payment breakdowns in under 2 seconds.
 2. Pre-Qualified WhatsApp Leads: Tap any WhatsApp button—it pre-fills the exact plot/project inquiry so your closers know what the buyer wants.

</xml_diff>